<commit_message>
Update GenCC Submission Spreadsheet template
🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/documents/GenCC Submission Spreadsheet.xlsx
+++ b/public/documents/GenCC Submission Spreadsheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lbabb/Development/gencc/gencc-sub/public/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2E1D078-F07F-2742-8AAA-5CB468963F6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C0DAF42-6AB4-8149-BA66-7C86F8F22FD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="129">
   <si>
     <t xml:space="preserve">REQUIRED Fields: These fields are required for the submission intake and records without these fields will be rejected. </t>
   </si>
@@ -182,9 +182,6 @@
     <t>Autosomal dominant inheritance</t>
   </si>
   <si>
-    <t>00001</t>
-  </si>
-  <si>
     <t>Lab123 Corp</t>
   </si>
   <si>
@@ -204,18 +201,6 @@
   </si>
   <si>
     <t>http://website.com/doc/something.pdf</t>
-  </si>
-  <si>
-    <t>HGNC:4321</t>
-  </si>
-  <si>
-    <t>ABC321</t>
-  </si>
-  <si>
-    <t>OMIM:123456</t>
-  </si>
-  <si>
-    <t>ZYX DISEASE</t>
   </si>
   <si>
     <t>http://www.website.com/something/12345</t>
@@ -419,19 +404,10 @@
     <t>GenCC Submission Sheet - Version 2</t>
   </si>
   <si>
-    <t>REQUIRED - The full url to where a visitor can access a public report/information (not in GenCC)</t>
-  </si>
-  <si>
     <t>REQUIRED for updates ONLY. This MUST be left blank for NEW submissions</t>
   </si>
   <si>
-    <t>SGC-0001</t>
-  </si>
-  <si>
     <t>PLEASE START SUBISSIONS IN THE NEXT ROW</t>
-  </si>
-  <si>
-    <t>SGC-0234</t>
   </si>
   <si>
     <t>VERSION2</t>
@@ -462,6 +438,18 @@
   </si>
   <si>
     <t>N</t>
+  </si>
+  <si>
+    <t>OPTIONAL - The full url to where a visitor can access a public report/information (not in GenCC)</t>
+  </si>
+  <si>
+    <t>GENCC:999999</t>
+  </si>
+  <si>
+    <t>SGC-999998</t>
+  </si>
+  <si>
+    <t>SGC-888888</t>
   </si>
 </sst>
 </file>
@@ -1023,7 +1011,7 @@
   <sheetData>
     <row r="1" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="B1" s="44"/>
       <c r="C1" s="1"/>
@@ -1163,7 +1151,7 @@
     </row>
     <row r="5" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="39" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="B5" s="46"/>
       <c r="C5" s="9"/>
@@ -1198,13 +1186,13 @@
     </row>
     <row r="6" spans="1:32" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A6" s="43" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="B6" s="47" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="C6" s="43" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="D6" s="12" t="s">
         <v>3</v>
@@ -1239,7 +1227,7 @@
       <c r="N6" s="40" t="s">
         <v>13</v>
       </c>
-      <c r="O6" s="40" t="s">
+      <c r="O6" s="13" t="s">
         <v>14</v>
       </c>
       <c r="P6" s="14" t="s">
@@ -1268,13 +1256,13 @@
     </row>
     <row r="7" spans="1:32" ht="187" customHeight="1" thickTop="1" x14ac:dyDescent="0.15">
       <c r="A7" s="15" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="B7" s="48" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="D7" s="16" t="s">
         <v>18</v>
@@ -1310,7 +1298,7 @@
         <v>28</v>
       </c>
       <c r="O7" s="18" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="P7" s="19" t="s">
         <v>29</v>
@@ -1373,11 +1361,11 @@
       <c r="AF8" s="28"/>
     </row>
     <row r="9" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" t="s">
-        <v>121</v>
+      <c r="A9" s="42" t="s">
+        <v>127</v>
       </c>
       <c r="B9" s="49" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="C9" s="29" t="s">
         <v>33</v>
@@ -1401,82 +1389,54 @@
         <v>39</v>
       </c>
       <c r="J9" s="29" t="s">
+        <v>126</v>
+      </c>
+      <c r="K9" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="K9" s="29" t="s">
+      <c r="L9" s="29" t="s">
         <v>41</v>
       </c>
-      <c r="L9" s="29" t="s">
+      <c r="M9" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="M9" s="29" t="s">
+      <c r="N9" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="N9" s="30" t="s">
+      <c r="O9" s="31"/>
+      <c r="P9" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="O9" s="31" t="s">
-        <v>52</v>
-      </c>
-      <c r="P9" s="32" t="s">
+      <c r="Q9" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="Q9" s="33" t="s">
+      <c r="R9" s="34" t="s">
         <v>46</v>
-      </c>
-      <c r="R9" s="34" t="s">
-        <v>47</v>
       </c>
       <c r="S9" s="35"/>
       <c r="T9" s="35"/>
     </row>
     <row r="10" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="42" t="s">
+        <v>128</v>
+      </c>
+      <c r="B10" s="49" t="s">
         <v>123</v>
       </c>
-      <c r="B10" s="49" t="s">
-        <v>131</v>
-      </c>
       <c r="C10" s="29"/>
-      <c r="D10" s="29" t="s">
-        <v>48</v>
-      </c>
-      <c r="E10" s="29" t="s">
-        <v>49</v>
-      </c>
-      <c r="F10" s="29" t="s">
-        <v>50</v>
-      </c>
-      <c r="G10" s="29" t="s">
-        <v>51</v>
-      </c>
-      <c r="H10" s="29" t="s">
-        <v>38</v>
-      </c>
-      <c r="I10" s="29" t="s">
-        <v>39</v>
-      </c>
-      <c r="J10" s="29" t="s">
-        <v>40</v>
-      </c>
-      <c r="K10" s="29" t="s">
-        <v>41</v>
-      </c>
-      <c r="L10" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="M10" s="29" t="s">
-        <v>43</v>
-      </c>
-      <c r="N10" s="30" t="s">
-        <v>44</v>
-      </c>
-      <c r="O10" s="31" t="s">
-        <v>52</v>
-      </c>
-      <c r="P10" s="32" t="s">
-        <v>45</v>
-      </c>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="29"/>
+      <c r="J10" s="29"/>
+      <c r="K10" s="29"/>
+      <c r="L10" s="29"/>
+      <c r="M10" s="29"/>
+      <c r="N10" s="30"/>
+      <c r="O10" s="31"/>
+      <c r="P10" s="32"/>
       <c r="Q10" s="33"/>
       <c r="R10" s="36"/>
       <c r="S10" s="35"/>
@@ -1484,19 +1444,19 @@
     </row>
     <row r="11" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B11" s="49" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="C11" s="29" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="D11" s="29" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="E11" s="29" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F11" s="29" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="G11" s="29"/>
       <c r="H11" s="29" t="s">
@@ -1506,36 +1466,36 @@
         <v>39</v>
       </c>
       <c r="J11" s="29" t="s">
+        <v>126</v>
+      </c>
+      <c r="K11" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="K11" s="29" t="s">
+      <c r="L11" s="29" t="s">
         <v>41</v>
       </c>
-      <c r="L11" s="29" t="s">
+      <c r="M11" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="M11" s="29" t="s">
+      <c r="N11" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="N11" s="30" t="s">
-        <v>44</v>
-      </c>
       <c r="O11" s="31" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="P11" s="32"/>
       <c r="Q11" s="33" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="R11" s="37" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="S11" s="35"/>
       <c r="T11" s="35"/>
     </row>
     <row r="12" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="22" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="B12" s="23"/>
       <c r="C12" s="22"/>
@@ -26063,12 +26023,12 @@
   <sheetData>
     <row r="1" spans="1:30" x14ac:dyDescent="0.15">
       <c r="A1" s="41" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="5" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -26110,106 +26070,106 @@
     </row>
     <row r="4" spans="1:30" ht="14.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.15">
       <c r="A4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="5" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B5" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="6" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B6" t="s">
         <v>71</v>
       </c>
-      <c r="B4" t="s">
+    </row>
+    <row r="7" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A7" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A5" t="s">
+      <c r="B7" t="s">
         <v>73</v>
       </c>
-      <c r="B5" t="s">
+    </row>
+    <row r="8" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A9" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A6" t="s">
+      <c r="B9" t="s">
         <v>75</v>
       </c>
-      <c r="B6" t="s">
+    </row>
+    <row r="10" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A10" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A7" t="s">
+      <c r="B10" t="s">
         <v>77</v>
       </c>
-      <c r="B7" t="s">
+    </row>
+    <row r="11" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A11" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A8" t="s">
-        <v>58</v>
-      </c>
-      <c r="B8" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A9" t="s">
+      <c r="B11" t="s">
         <v>79</v>
       </c>
-      <c r="B9" t="s">
+    </row>
+    <row r="12" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A12" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A10" t="s">
+      <c r="B12" t="s">
         <v>81</v>
       </c>
-      <c r="B10" t="s">
+    </row>
+    <row r="13" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A13" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A11" t="s">
+      <c r="B13" t="s">
         <v>83</v>
       </c>
-      <c r="B11" t="s">
+    </row>
+    <row r="14" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A14" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A12" t="s">
+      <c r="B14" t="s">
         <v>85</v>
       </c>
-      <c r="B12" t="s">
+    </row>
+    <row r="15" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A15" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A13" t="s">
+      <c r="B15" t="s">
         <v>87</v>
       </c>
-      <c r="B13" t="s">
+    </row>
+    <row r="16" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A16" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A14" t="s">
+      <c r="B16" t="s">
         <v>89</v>
-      </c>
-      <c r="B14" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A15" t="s">
-        <v>91</v>
-      </c>
-      <c r="B15" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A16" t="s">
-        <v>93</v>
-      </c>
-      <c r="B16" t="s">
-        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -26229,12 +26189,12 @@
   <sheetData>
     <row r="1" spans="1:30" x14ac:dyDescent="0.15">
       <c r="A1" s="41" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="5" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -26276,74 +26236,74 @@
     </row>
     <row r="4" spans="1:30" ht="14.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.15">
       <c r="A4" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="B4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:30" x14ac:dyDescent="0.15">
       <c r="A5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B6" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="7" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A7" t="s">
+        <v>62</v>
+      </c>
+      <c r="B7" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="8" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A8" t="s">
+        <v>92</v>
+      </c>
+      <c r="B8" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="9" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B9" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="10" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A10" t="s">
+        <v>96</v>
+      </c>
+      <c r="B10" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="11" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A11" t="s">
         <v>60</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B11" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A6" t="s">
-        <v>62</v>
-      </c>
-      <c r="B6" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A7" t="s">
-        <v>67</v>
-      </c>
-      <c r="B7" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A8" t="s">
-        <v>97</v>
-      </c>
-      <c r="B8" t="s">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A12" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A9" t="s">
+      <c r="B12" t="s">
         <v>99</v>
-      </c>
-      <c r="B9" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A10" t="s">
-        <v>101</v>
-      </c>
-      <c r="B10" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A11" t="s">
-        <v>65</v>
-      </c>
-      <c r="B11" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A12" t="s">
-        <v>103</v>
-      </c>
-      <c r="B12" t="s">
-        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -26363,12 +26323,12 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A1" s="41" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A2" s="5" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="B2" s="6"/>
     </row>
@@ -26390,50 +26350,50 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A6" t="s">
+        <v>103</v>
+      </c>
+      <c r="B6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A7" t="s">
+        <v>105</v>
+      </c>
+      <c r="B7" t="s">
         <v>106</v>
       </c>
-      <c r="B5" t="s">
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A8" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A6" t="s">
+      <c r="B8" t="s">
         <v>108</v>
       </c>
-      <c r="B6" t="s">
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A9" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A7" t="s">
+      <c r="B9" t="s">
         <v>110</v>
       </c>
-      <c r="B7" t="s">
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A10" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A8" t="s">
+      <c r="B10" t="s">
         <v>112</v>
-      </c>
-      <c r="B8" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A9" t="s">
-        <v>114</v>
-      </c>
-      <c r="B9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A10" t="s">
-        <v>116</v>
-      </c>
-      <c r="B10" t="s">
-        <v>117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update GenCC Submission Spreadsheet template (#65)
🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-authored-by: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/documents/GenCC Submission Spreadsheet.xlsx
+++ b/public/documents/GenCC Submission Spreadsheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lbabb/Development/gencc/gencc-sub/public/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2E1D078-F07F-2742-8AAA-5CB468963F6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C0DAF42-6AB4-8149-BA66-7C86F8F22FD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="129">
   <si>
     <t xml:space="preserve">REQUIRED Fields: These fields are required for the submission intake and records without these fields will be rejected. </t>
   </si>
@@ -182,9 +182,6 @@
     <t>Autosomal dominant inheritance</t>
   </si>
   <si>
-    <t>00001</t>
-  </si>
-  <si>
     <t>Lab123 Corp</t>
   </si>
   <si>
@@ -204,18 +201,6 @@
   </si>
   <si>
     <t>http://website.com/doc/something.pdf</t>
-  </si>
-  <si>
-    <t>HGNC:4321</t>
-  </si>
-  <si>
-    <t>ABC321</t>
-  </si>
-  <si>
-    <t>OMIM:123456</t>
-  </si>
-  <si>
-    <t>ZYX DISEASE</t>
   </si>
   <si>
     <t>http://www.website.com/something/12345</t>
@@ -419,19 +404,10 @@
     <t>GenCC Submission Sheet - Version 2</t>
   </si>
   <si>
-    <t>REQUIRED - The full url to where a visitor can access a public report/information (not in GenCC)</t>
-  </si>
-  <si>
     <t>REQUIRED for updates ONLY. This MUST be left blank for NEW submissions</t>
   </si>
   <si>
-    <t>SGC-0001</t>
-  </si>
-  <si>
     <t>PLEASE START SUBISSIONS IN THE NEXT ROW</t>
-  </si>
-  <si>
-    <t>SGC-0234</t>
   </si>
   <si>
     <t>VERSION2</t>
@@ -462,6 +438,18 @@
   </si>
   <si>
     <t>N</t>
+  </si>
+  <si>
+    <t>OPTIONAL - The full url to where a visitor can access a public report/information (not in GenCC)</t>
+  </si>
+  <si>
+    <t>GENCC:999999</t>
+  </si>
+  <si>
+    <t>SGC-999998</t>
+  </si>
+  <si>
+    <t>SGC-888888</t>
   </si>
 </sst>
 </file>
@@ -1023,7 +1011,7 @@
   <sheetData>
     <row r="1" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="B1" s="44"/>
       <c r="C1" s="1"/>
@@ -1163,7 +1151,7 @@
     </row>
     <row r="5" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="39" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="B5" s="46"/>
       <c r="C5" s="9"/>
@@ -1198,13 +1186,13 @@
     </row>
     <row r="6" spans="1:32" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A6" s="43" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="B6" s="47" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="C6" s="43" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="D6" s="12" t="s">
         <v>3</v>
@@ -1239,7 +1227,7 @@
       <c r="N6" s="40" t="s">
         <v>13</v>
       </c>
-      <c r="O6" s="40" t="s">
+      <c r="O6" s="13" t="s">
         <v>14</v>
       </c>
       <c r="P6" s="14" t="s">
@@ -1268,13 +1256,13 @@
     </row>
     <row r="7" spans="1:32" ht="187" customHeight="1" thickTop="1" x14ac:dyDescent="0.15">
       <c r="A7" s="15" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="B7" s="48" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="D7" s="16" t="s">
         <v>18</v>
@@ -1310,7 +1298,7 @@
         <v>28</v>
       </c>
       <c r="O7" s="18" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="P7" s="19" t="s">
         <v>29</v>
@@ -1373,11 +1361,11 @@
       <c r="AF8" s="28"/>
     </row>
     <row r="9" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" t="s">
-        <v>121</v>
+      <c r="A9" s="42" t="s">
+        <v>127</v>
       </c>
       <c r="B9" s="49" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="C9" s="29" t="s">
         <v>33</v>
@@ -1401,82 +1389,54 @@
         <v>39</v>
       </c>
       <c r="J9" s="29" t="s">
+        <v>126</v>
+      </c>
+      <c r="K9" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="K9" s="29" t="s">
+      <c r="L9" s="29" t="s">
         <v>41</v>
       </c>
-      <c r="L9" s="29" t="s">
+      <c r="M9" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="M9" s="29" t="s">
+      <c r="N9" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="N9" s="30" t="s">
+      <c r="O9" s="31"/>
+      <c r="P9" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="O9" s="31" t="s">
-        <v>52</v>
-      </c>
-      <c r="P9" s="32" t="s">
+      <c r="Q9" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="Q9" s="33" t="s">
+      <c r="R9" s="34" t="s">
         <v>46</v>
-      </c>
-      <c r="R9" s="34" t="s">
-        <v>47</v>
       </c>
       <c r="S9" s="35"/>
       <c r="T9" s="35"/>
     </row>
     <row r="10" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="42" t="s">
+        <v>128</v>
+      </c>
+      <c r="B10" s="49" t="s">
         <v>123</v>
       </c>
-      <c r="B10" s="49" t="s">
-        <v>131</v>
-      </c>
       <c r="C10" s="29"/>
-      <c r="D10" s="29" t="s">
-        <v>48</v>
-      </c>
-      <c r="E10" s="29" t="s">
-        <v>49</v>
-      </c>
-      <c r="F10" s="29" t="s">
-        <v>50</v>
-      </c>
-      <c r="G10" s="29" t="s">
-        <v>51</v>
-      </c>
-      <c r="H10" s="29" t="s">
-        <v>38</v>
-      </c>
-      <c r="I10" s="29" t="s">
-        <v>39</v>
-      </c>
-      <c r="J10" s="29" t="s">
-        <v>40</v>
-      </c>
-      <c r="K10" s="29" t="s">
-        <v>41</v>
-      </c>
-      <c r="L10" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="M10" s="29" t="s">
-        <v>43</v>
-      </c>
-      <c r="N10" s="30" t="s">
-        <v>44</v>
-      </c>
-      <c r="O10" s="31" t="s">
-        <v>52</v>
-      </c>
-      <c r="P10" s="32" t="s">
-        <v>45</v>
-      </c>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="29"/>
+      <c r="J10" s="29"/>
+      <c r="K10" s="29"/>
+      <c r="L10" s="29"/>
+      <c r="M10" s="29"/>
+      <c r="N10" s="30"/>
+      <c r="O10" s="31"/>
+      <c r="P10" s="32"/>
       <c r="Q10" s="33"/>
       <c r="R10" s="36"/>
       <c r="S10" s="35"/>
@@ -1484,19 +1444,19 @@
     </row>
     <row r="11" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B11" s="49" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="C11" s="29" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="D11" s="29" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="E11" s="29" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F11" s="29" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="G11" s="29"/>
       <c r="H11" s="29" t="s">
@@ -1506,36 +1466,36 @@
         <v>39</v>
       </c>
       <c r="J11" s="29" t="s">
+        <v>126</v>
+      </c>
+      <c r="K11" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="K11" s="29" t="s">
+      <c r="L11" s="29" t="s">
         <v>41</v>
       </c>
-      <c r="L11" s="29" t="s">
+      <c r="M11" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="M11" s="29" t="s">
+      <c r="N11" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="N11" s="30" t="s">
-        <v>44</v>
-      </c>
       <c r="O11" s="31" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="P11" s="32"/>
       <c r="Q11" s="33" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="R11" s="37" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="S11" s="35"/>
       <c r="T11" s="35"/>
     </row>
     <row r="12" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="22" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="B12" s="23"/>
       <c r="C12" s="22"/>
@@ -26063,12 +26023,12 @@
   <sheetData>
     <row r="1" spans="1:30" x14ac:dyDescent="0.15">
       <c r="A1" s="41" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="5" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -26110,106 +26070,106 @@
     </row>
     <row r="4" spans="1:30" ht="14.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.15">
       <c r="A4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="5" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B5" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="6" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B6" t="s">
         <v>71</v>
       </c>
-      <c r="B4" t="s">
+    </row>
+    <row r="7" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A7" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A5" t="s">
+      <c r="B7" t="s">
         <v>73</v>
       </c>
-      <c r="B5" t="s">
+    </row>
+    <row r="8" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A9" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A6" t="s">
+      <c r="B9" t="s">
         <v>75</v>
       </c>
-      <c r="B6" t="s">
+    </row>
+    <row r="10" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A10" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A7" t="s">
+      <c r="B10" t="s">
         <v>77</v>
       </c>
-      <c r="B7" t="s">
+    </row>
+    <row r="11" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A11" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A8" t="s">
-        <v>58</v>
-      </c>
-      <c r="B8" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A9" t="s">
+      <c r="B11" t="s">
         <v>79</v>
       </c>
-      <c r="B9" t="s">
+    </row>
+    <row r="12" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A12" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A10" t="s">
+      <c r="B12" t="s">
         <v>81</v>
       </c>
-      <c r="B10" t="s">
+    </row>
+    <row r="13" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A13" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A11" t="s">
+      <c r="B13" t="s">
         <v>83</v>
       </c>
-      <c r="B11" t="s">
+    </row>
+    <row r="14" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A14" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A12" t="s">
+      <c r="B14" t="s">
         <v>85</v>
       </c>
-      <c r="B12" t="s">
+    </row>
+    <row r="15" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A15" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A13" t="s">
+      <c r="B15" t="s">
         <v>87</v>
       </c>
-      <c r="B13" t="s">
+    </row>
+    <row r="16" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A16" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A14" t="s">
+      <c r="B16" t="s">
         <v>89</v>
-      </c>
-      <c r="B14" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A15" t="s">
-        <v>91</v>
-      </c>
-      <c r="B15" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A16" t="s">
-        <v>93</v>
-      </c>
-      <c r="B16" t="s">
-        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -26229,12 +26189,12 @@
   <sheetData>
     <row r="1" spans="1:30" x14ac:dyDescent="0.15">
       <c r="A1" s="41" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="5" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -26276,74 +26236,74 @@
     </row>
     <row r="4" spans="1:30" ht="14.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.15">
       <c r="A4" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="B4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:30" x14ac:dyDescent="0.15">
       <c r="A5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B6" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="7" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A7" t="s">
+        <v>62</v>
+      </c>
+      <c r="B7" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="8" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A8" t="s">
+        <v>92</v>
+      </c>
+      <c r="B8" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="9" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B9" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="10" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A10" t="s">
+        <v>96</v>
+      </c>
+      <c r="B10" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="11" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A11" t="s">
         <v>60</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B11" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A6" t="s">
-        <v>62</v>
-      </c>
-      <c r="B6" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A7" t="s">
-        <v>67</v>
-      </c>
-      <c r="B7" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A8" t="s">
-        <v>97</v>
-      </c>
-      <c r="B8" t="s">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A12" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A9" t="s">
+      <c r="B12" t="s">
         <v>99</v>
-      </c>
-      <c r="B9" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A10" t="s">
-        <v>101</v>
-      </c>
-      <c r="B10" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A11" t="s">
-        <v>65</v>
-      </c>
-      <c r="B11" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A12" t="s">
-        <v>103</v>
-      </c>
-      <c r="B12" t="s">
-        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -26363,12 +26323,12 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A1" s="41" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A2" s="5" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="B2" s="6"/>
     </row>
@@ -26390,50 +26350,50 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A6" t="s">
+        <v>103</v>
+      </c>
+      <c r="B6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A7" t="s">
+        <v>105</v>
+      </c>
+      <c r="B7" t="s">
         <v>106</v>
       </c>
-      <c r="B5" t="s">
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A8" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A6" t="s">
+      <c r="B8" t="s">
         <v>108</v>
       </c>
-      <c r="B6" t="s">
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A9" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A7" t="s">
+      <c r="B9" t="s">
         <v>110</v>
       </c>
-      <c r="B7" t="s">
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A10" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A8" t="s">
+      <c r="B10" t="s">
         <v>112</v>
-      </c>
-      <c r="B8" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A9" t="s">
-        <v>114</v>
-      </c>
-      <c r="B9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A10" t="s">
-        <v>116</v>
-      </c>
-      <c r="B10" t="s">
-        <v>117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corrected and completed the HELP-Submitter Ids sheet on the submission template that is downloadable.
</commit_message>
<xml_diff>
--- a/public/documents/GenCC Submission Spreadsheet.xlsx
+++ b/public/documents/GenCC Submission Spreadsheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lbabb/Development/gencc/gencc-sub/public/documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lbabb/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C0DAF42-6AB4-8149-BA66-7C86F8F22FD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDC6E0E8-F514-A940-B935-560F0EA80A4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="141">
   <si>
     <t xml:space="preserve">REQUIRED Fields: These fields are required for the submission intake and records without these fields will be rejected. </t>
   </si>
@@ -323,9 +323,6 @@
     <t>GENCC:000112</t>
   </si>
   <si>
-    <t>TGMI</t>
-  </si>
-  <si>
     <t>GENCC:000113</t>
   </si>
   <si>
@@ -450,6 +447,45 @@
   </si>
   <si>
     <t>SGC-888888</t>
+  </si>
+  <si>
+    <t>Franklin by Genoox</t>
+  </si>
+  <si>
+    <t>King Faisal Specialist Hospital and Research Center</t>
+  </si>
+  <si>
+    <t>Broad Center for Mendelian Genomics</t>
+  </si>
+  <si>
+    <t>Baylor College of Medicine Research Center</t>
+  </si>
+  <si>
+    <t>GENCC:000114</t>
+  </si>
+  <si>
+    <t>GENCC:000115</t>
+  </si>
+  <si>
+    <t>GENCC:000116</t>
+  </si>
+  <si>
+    <t>GENCC:000117</t>
+  </si>
+  <si>
+    <t>LiferaOmics</t>
+  </si>
+  <si>
+    <t>University of Washington Center for Rare Disease Reseaerch (UW-CRDR)</t>
+  </si>
+  <si>
+    <t>Stanford Center for Undiagnosed Disease</t>
+  </si>
+  <si>
+    <t>GENCC:000118</t>
+  </si>
+  <si>
+    <t>GENCC:000119</t>
   </si>
 </sst>
 </file>
@@ -1011,7 +1047,7 @@
   <sheetData>
     <row r="1" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B1" s="44"/>
       <c r="C1" s="1"/>
@@ -1151,7 +1187,7 @@
     </row>
     <row r="5" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="39" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B5" s="46"/>
       <c r="C5" s="9"/>
@@ -1186,13 +1222,13 @@
     </row>
     <row r="6" spans="1:32" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A6" s="43" t="s">
+        <v>118</v>
+      </c>
+      <c r="B6" s="47" t="s">
         <v>119</v>
       </c>
-      <c r="B6" s="47" t="s">
-        <v>120</v>
-      </c>
       <c r="C6" s="43" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D6" s="12" t="s">
         <v>3</v>
@@ -1256,13 +1292,13 @@
     </row>
     <row r="7" spans="1:32" ht="187" customHeight="1" thickTop="1" x14ac:dyDescent="0.15">
       <c r="A7" s="15" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B7" s="48" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D7" s="16" t="s">
         <v>18</v>
@@ -1298,7 +1334,7 @@
         <v>28</v>
       </c>
       <c r="O7" s="18" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="P7" s="19" t="s">
         <v>29</v>
@@ -1362,10 +1398,10 @@
     </row>
     <row r="9" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="42" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B9" s="49" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C9" s="29" t="s">
         <v>33</v>
@@ -1389,7 +1425,7 @@
         <v>39</v>
       </c>
       <c r="J9" s="29" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="K9" s="29" t="s">
         <v>40</v>
@@ -1418,10 +1454,10 @@
     </row>
     <row r="10" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="42" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B10" s="49" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C10" s="29"/>
       <c r="D10" s="29"/>
@@ -1444,7 +1480,7 @@
     </row>
     <row r="11" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B11" s="49" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C11" s="29" t="s">
         <v>48</v>
@@ -1466,7 +1502,7 @@
         <v>39</v>
       </c>
       <c r="J11" s="29" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="K11" s="29" t="s">
         <v>40</v>
@@ -1495,7 +1531,7 @@
     </row>
     <row r="12" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="22" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B12" s="23"/>
       <c r="C12" s="22"/>
@@ -26014,7 +26050,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:AD16"/>
+  <dimension ref="A1:AD23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="20.5" customWidth="1"/>
@@ -26160,19 +26196,71 @@
       <c r="A15" t="s">
         <v>86</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="42" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="16" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A16" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A16" t="s">
-        <v>88</v>
+      <c r="B16" s="42" t="s">
+        <v>128</v>
       </c>
-      <c r="B16" t="s">
-        <v>89</v>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A17" t="s">
+        <v>132</v>
       </c>
+      <c r="B17" s="42" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A18" t="s">
+        <v>133</v>
+      </c>
+      <c r="B18" s="42" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A19" t="s">
+        <v>134</v>
+      </c>
+      <c r="B19" s="42" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A20" t="s">
+        <v>135</v>
+      </c>
+      <c r="B20" s="42" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A21" t="s">
+        <v>139</v>
+      </c>
+      <c r="B21" s="42" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A22" t="s">
+        <v>140</v>
+      </c>
+      <c r="B22" s="42" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="B23" s="42"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="17" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -26189,12 +26277,12 @@
   <sheetData>
     <row r="1" spans="1:30" x14ac:dyDescent="0.15">
       <c r="A1" s="41" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -26268,26 +26356,26 @@
     </row>
     <row r="8" spans="1:30" x14ac:dyDescent="0.15">
       <c r="A8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B8" t="s">
         <v>92</v>
       </c>
-      <c r="B8" t="s">
+    </row>
+    <row r="9" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A9" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A9" t="s">
+      <c r="B9" t="s">
         <v>94</v>
       </c>
-      <c r="B9" t="s">
+    </row>
+    <row r="10" spans="1:30" x14ac:dyDescent="0.15">
+      <c r="A10" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.15">
-      <c r="A10" t="s">
+      <c r="B10" t="s">
         <v>96</v>
-      </c>
-      <c r="B10" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="11" spans="1:30" x14ac:dyDescent="0.15">
@@ -26300,10 +26388,10 @@
     </row>
     <row r="12" spans="1:30" x14ac:dyDescent="0.15">
       <c r="A12" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B12" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -26323,12 +26411,12 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A1" s="41" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A2" s="5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B2" s="6"/>
     </row>
@@ -26350,50 +26438,50 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A5" t="s">
+        <v>100</v>
+      </c>
+      <c r="B5" t="s">
         <v>101</v>
       </c>
-      <c r="B5" t="s">
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A6" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A6" t="s">
+      <c r="B6" t="s">
         <v>103</v>
       </c>
-      <c r="B6" t="s">
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A7" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A7" t="s">
+      <c r="B7" t="s">
         <v>105</v>
       </c>
-      <c r="B7" t="s">
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A8" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A8" t="s">
+      <c r="B8" t="s">
         <v>107</v>
       </c>
-      <c r="B8" t="s">
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A9" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A9" t="s">
+      <c r="B9" t="s">
         <v>109</v>
       </c>
-      <c r="B9" t="s">
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A10" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A10" t="s">
+      <c r="B10" t="s">
         <v>111</v>
-      </c>
-      <c r="B10" t="s">
-        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>